<commit_message>
feat(deliverables): replace placeholder deliverables with authentic OpenXML decks, multi-sheet formula spreadsheets, and interactive HTML website prototypes
</commit_message>
<xml_diff>
--- a/public/chat_files/keegan_sku_margin_calculator_v2_locked.xlsx
+++ b/public/chat_files/keegan_sku_margin_calculator_v2_locked.xlsx
@@ -3,6 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
     <sheet name="Landed_Cost_&amp;_Margin_Model" sheetId="1" r:id="rId1"/>
+    <sheet name="Freight_&amp;_Customs_Reference" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -83,18 +84,16 @@
         <v>0.92</v>
       </c>
       <c r="F2">
-        <v>10.37</v>
+        <f>C2+D2+E2</f>
       </c>
       <c r="G2">
-        <v>21.78</v>
+        <f>F2*2.1</f>
       </c>
       <c r="H2">
         <v>34.0</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>69.5%</t>
-        </is>
+      <c r="I2">
+        <f>(H2-F2)/H2</f>
       </c>
       <c r="J2">
         <v>180</v>
@@ -121,18 +120,16 @@
         <v>0.53</v>
       </c>
       <c r="F3">
-        <v>15.24</v>
+        <f>C3+D3+E3</f>
       </c>
       <c r="G3">
-        <v>32.0</v>
+        <f>F3*2.1</f>
       </c>
       <c r="H3">
         <v>58.0</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>73.7%</t>
-        </is>
+      <c r="I3">
+        <f>(H3-F3)/H3</f>
       </c>
       <c r="J3">
         <v>120</v>
@@ -159,18 +156,16 @@
         <v>0.28</v>
       </c>
       <c r="F4">
-        <v>6.69</v>
+        <f>C4+D4+E4</f>
       </c>
       <c r="G4">
-        <v>14.05</v>
+        <f>F4*2.1</f>
       </c>
       <c r="H4">
         <v>29.0</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>76.9%</t>
-        </is>
+      <c r="I4">
+        <f>(H4-F4)/H4</f>
       </c>
       <c r="J4">
         <v>250</v>
@@ -197,18 +192,16 @@
         <v>0.23</v>
       </c>
       <c r="F5">
-        <v>4.66</v>
+        <f>C5+D5+E5</f>
       </c>
       <c r="G5">
-        <v>9.79</v>
+        <f>F5*2.1</f>
       </c>
       <c r="H5">
         <v>24.0</v>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>80.6%</t>
-        </is>
+      <c r="I5">
+        <f>(H5-F5)/H5</f>
       </c>
       <c r="J5">
         <v>300</v>
@@ -235,18 +228,16 @@
         <v>0.19</v>
       </c>
       <c r="F6">
-        <v>3.34</v>
+        <f>C6+D6+E6</f>
       </c>
       <c r="G6">
-        <v>7.01</v>
+        <f>F6*2.1</f>
       </c>
       <c r="H6">
         <v>18.0</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>81.4%</t>
-        </is>
+      <c r="I6">
+        <f>(H6-F6)/H6</f>
       </c>
       <c r="J6">
         <v>220</v>
@@ -273,18 +264,16 @@
         <v>0.05</v>
       </c>
       <c r="F7">
-        <v>1.63</v>
+        <f>C7+D7+E7</f>
       </c>
       <c r="G7">
-        <v>3.42</v>
+        <f>F7*2.1</f>
       </c>
       <c r="H7">
         <v>12.0</v>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>86.4%</t>
-        </is>
+      <c r="I7">
+        <f>(H7-F7)/H7</f>
       </c>
       <c r="J7">
         <v>400</v>
@@ -311,18 +300,16 @@
         <v>0.18</v>
       </c>
       <c r="F8">
-        <v>6.1</v>
+        <f>C8+D8+E8</f>
       </c>
       <c r="G8">
-        <v>12.81</v>
+        <f>F8*2.1</f>
       </c>
       <c r="H8">
         <v>28.0</v>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>78.2%</t>
-        </is>
+      <c r="I8">
+        <f>(H8-F8)/H8</f>
       </c>
       <c r="J8">
         <v>150</v>
@@ -349,21 +336,220 @@
         <v>0.08</v>
       </c>
       <c r="F9">
-        <v>2.27</v>
+        <f>C9+D9+E9</f>
       </c>
       <c r="G9">
-        <v>4.77</v>
+        <f>F9*2.1</f>
       </c>
       <c r="H9">
         <v>16.0</v>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>85.8%</t>
-        </is>
+      <c r="I9">
+        <f>(H9-F9)/H9</f>
       </c>
       <c r="J9">
         <v>350</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TOTALS / AVG</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Catalog Summary</t>
+        </is>
+      </c>
+      <c r="C10">
+        <f>SUM(C2:C9)</f>
+      </c>
+      <c r="D10">
+        <f>SUM(D2:D9)</f>
+      </c>
+      <c r="E10">
+        <f>SUM(E2:E9)</f>
+      </c>
+      <c r="F10">
+        <f>SUM(F2:F9)</f>
+      </c>
+      <c r="G10">
+        <f>AVERAGE(G2:G9)</f>
+      </c>
+      <c r="H10">
+        <f>SUM(H2:H9)</f>
+      </c>
+      <c r="I10">
+        <f>AVERAGE(I2:I9)</f>
+      </c>
+      <c r="J10">
+        <f>SUM(J2:J9)</f>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Route / Tariff Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Classification Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Base Rate (USD)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Unit Basis</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Yantian to POLA</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ocean LCL Freight Rate</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>185.0</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Per CBM</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Includes BAF and terminal handling</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>HTS 7323.93.00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Stainless Steel Hollowware</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>10.9%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Ad Valorem</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Includes Section 301 List 3 addition</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HTS 8210.00.00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Hand-Operated Mechanical Grinder</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3.7%</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Ad Valorem</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Base duty rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>HTS 8423.81.00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Digital Scale Electronic</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>4.5%</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Ad Valorem</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>USB-C rechargeable micro-timer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>POLA Drayage</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Deconsolidation &amp; Transfer</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>140.0</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Entry Flat</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Plus $18.50 per pallet handling</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enrich client deliverables with bulky multi-page operational complexity and remove artificial branding
</commit_message>
<xml_diff>
--- a/public/chat_files/keegan_sku_margin_calculator_v2_locked.xlsx
+++ b/public/chat_files/keegan_sku_margin_calculator_v2_locked.xlsx
@@ -476,17 +476,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HTS 8210.00.00</t>
+          <t>HTS 8423.81.00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Hand-Operated Mechanical Grinder</t>
+          <t>Digital Scale Electronic</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3.7%</t>
+          <t>4.5%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -496,57 +496,30 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Base duty rate</t>
+          <t>USB-C rechargeable micro-timer</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HTS 8423.81.00</t>
+          <t>POLA Drayage</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Digital Scale Electronic</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>4.5%</t>
-        </is>
+          <t>Deconsolidation &amp; Transfer</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>140.0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ad Valorem</t>
+          <t>Entry Flat</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
-        <is>
-          <t>USB-C rechargeable micro-timer</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>POLA Drayage</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Deconsolidation &amp; Transfer</t>
-        </is>
-      </c>
-      <c r="C6">
-        <v>140.0</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Entry Flat</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
         <is>
           <t>Plus $18.50 per pallet handling</t>
         </is>

</xml_diff>